<commit_message>
Missing labels for roles
</commit_message>
<xml_diff>
--- a/owlcms/src/main/resources/templates/protocol/SnCJTot-A4.xlsx
+++ b/owlcms/src/main/resources/templates/protocol/SnCJTot-A4.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lamyj\git\owlcms4\owlcms\src\main\resources\templates\protocol\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E451621D-60B0-495E-9AAC-7B440ABFA23B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23CB1B51-7582-462F-9219-0CD1C9BB636C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2730" yWindow="1665" windowWidth="24615" windowHeight="11310" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Results" sheetId="1" r:id="rId1"/>
@@ -156,7 +156,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="90">
   <si>
     <t>${l.lotNumber}</t>
   </si>
@@ -417,6 +417,15 @@
   </si>
   <si>
     <t>${session.announcerAsTO} ${session.announcerAsTO.federationId}</t>
+  </si>
+  <si>
+    <t>${t.get("Marshall")}</t>
+  </si>
+  <si>
+    <t>${t.get("Timekeeper")}</t>
+  </si>
+  <si>
+    <t>${t.get("Results.Controller")}</t>
   </si>
 </sst>
 </file>
@@ -1112,7 +1121,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="117">
+  <cellXfs count="119">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1370,36 +1379,6 @@
     </xf>
     <xf numFmtId="1" fontId="33" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1427,6 +1406,12 @@
     <xf numFmtId="0" fontId="9" fillId="12" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
@@ -1434,6 +1419,36 @@
     <xf numFmtId="0" fontId="0" fillId="12" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="19">
@@ -2041,63 +2056,63 @@
     </row>
     <row r="5" spans="1:24" ht="6" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="6" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="98" t="s">
+      <c r="A6" s="111" t="s">
         <v>38</v>
       </c>
-      <c r="B6" s="98" t="s">
+      <c r="B6" s="111" t="s">
         <v>42</v>
       </c>
-      <c r="C6" s="100" t="s">
+      <c r="C6" s="113" t="s">
         <v>30</v>
       </c>
-      <c r="D6" s="102" t="s">
+      <c r="D6" s="115" t="s">
         <v>31</v>
       </c>
-      <c r="E6" s="104" t="s">
+      <c r="E6" s="107" t="s">
         <v>32</v>
       </c>
-      <c r="F6" s="104" t="s">
+      <c r="F6" s="107" t="s">
         <v>33</v>
       </c>
-      <c r="G6" s="104" t="s">
+      <c r="G6" s="107" t="s">
         <v>34</v>
       </c>
-      <c r="H6" s="104" t="s">
+      <c r="H6" s="107" t="s">
         <v>35</v>
       </c>
-      <c r="I6" s="115" t="s">
+      <c r="I6" s="109" t="s">
         <v>36</v>
       </c>
-      <c r="J6" s="116"/>
-      <c r="K6" s="116"/>
-      <c r="L6" s="116"/>
-      <c r="M6" s="116"/>
-      <c r="N6" s="115" t="s">
+      <c r="J6" s="110"/>
+      <c r="K6" s="110"/>
+      <c r="L6" s="110"/>
+      <c r="M6" s="110"/>
+      <c r="N6" s="109" t="s">
         <v>37</v>
       </c>
-      <c r="O6" s="116"/>
-      <c r="P6" s="116"/>
-      <c r="Q6" s="116"/>
-      <c r="R6" s="116"/>
-      <c r="S6" s="113" t="s">
+      <c r="O6" s="110"/>
+      <c r="P6" s="110"/>
+      <c r="Q6" s="110"/>
+      <c r="R6" s="110"/>
+      <c r="S6" s="105" t="s">
         <v>39</v>
       </c>
-      <c r="T6" s="114"/>
-      <c r="U6" s="106" t="s">
+      <c r="T6" s="106"/>
+      <c r="U6" s="98" t="s">
         <v>76</v>
       </c>
-      <c r="V6" s="107"/>
+      <c r="V6" s="99"/>
       <c r="X6"/>
     </row>
     <row r="7" spans="1:24" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="99"/>
-      <c r="B7" s="99"/>
-      <c r="C7" s="101"/>
-      <c r="D7" s="103"/>
-      <c r="E7" s="105"/>
-      <c r="F7" s="105"/>
-      <c r="G7" s="105"/>
-      <c r="H7" s="105"/>
+      <c r="A7" s="112"/>
+      <c r="B7" s="112"/>
+      <c r="C7" s="114"/>
+      <c r="D7" s="116"/>
+      <c r="E7" s="108"/>
+      <c r="F7" s="108"/>
+      <c r="G7" s="108"/>
+      <c r="H7" s="108"/>
       <c r="I7" s="47">
         <v>1</v>
       </c>
@@ -2134,8 +2149,8 @@
       <c r="T7" s="49" t="s">
         <v>40</v>
       </c>
-      <c r="U7" s="108"/>
-      <c r="V7" s="109"/>
+      <c r="U7" s="100"/>
+      <c r="V7" s="101"/>
     </row>
     <row r="8" spans="1:24" s="11" customFormat="1" ht="7.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="38"/>
@@ -2238,10 +2253,10 @@
       <c r="T10" s="59" t="s">
         <v>46</v>
       </c>
-      <c r="U10" s="110" t="s">
+      <c r="U10" s="102" t="s">
         <v>77</v>
       </c>
-      <c r="V10" s="111"/>
+      <c r="V10" s="103"/>
     </row>
     <row r="11" spans="1:24" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11"/>
@@ -2398,12 +2413,19 @@
         <v>86</v>
       </c>
       <c r="D17" s="85"/>
+      <c r="E17" s="117" t="s">
+        <v>87</v>
+      </c>
       <c r="F17" s="84" t="s">
         <v>78</v>
       </c>
       <c r="G17" s="85"/>
       <c r="H17" s="85"/>
       <c r="I17" s="85"/>
+      <c r="J17" s="104" t="s">
+        <v>88</v>
+      </c>
+      <c r="K17" s="104"/>
       <c r="L17" s="84" t="s">
         <v>79</v>
       </c>
@@ -2411,6 +2433,10 @@
       <c r="N17" s="85"/>
       <c r="O17" s="85"/>
       <c r="P17" s="86"/>
+      <c r="Q17" s="118" t="s">
+        <v>89</v>
+      </c>
+      <c r="R17" s="118"/>
       <c r="S17" s="84" t="s">
         <v>80</v>
       </c>
@@ -2420,21 +2446,23 @@
       <c r="W17"/>
       <c r="X17" s="85"/>
     </row>
-    <row r="18" spans="1:24" s="89" customFormat="1" ht="11.25" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:24" s="89" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="87"/>
       <c r="B18" s="88"/>
       <c r="D18" s="90"/>
-      <c r="E18" s="91"/>
+      <c r="E18" s="117"/>
       <c r="F18" s="92"/>
       <c r="G18" s="90"/>
       <c r="I18" s="87"/>
-      <c r="K18" s="91"/>
+      <c r="J18" s="104"/>
+      <c r="K18" s="104"/>
       <c r="L18" s="90"/>
       <c r="M18" s="90"/>
       <c r="N18" s="90"/>
       <c r="O18" s="90"/>
       <c r="P18" s="90"/>
-      <c r="Q18" s="87"/>
+      <c r="Q18" s="118"/>
+      <c r="R18" s="118"/>
       <c r="S18" s="90"/>
       <c r="T18" s="90"/>
       <c r="U18" s="90"/>
@@ -2448,10 +2476,10 @@
       <c r="E19" s="94"/>
       <c r="F19" s="95"/>
       <c r="I19" s="1"/>
-      <c r="J19" s="112" t="s">
+      <c r="J19" s="104" t="s">
         <v>69</v>
       </c>
-      <c r="K19" s="112"/>
+      <c r="K19" s="104"/>
       <c r="M19"/>
       <c r="N19" s="1"/>
       <c r="O19" s="8"/>
@@ -2479,8 +2507,8 @@
       <c r="G20" s="85"/>
       <c r="H20" s="85"/>
       <c r="I20" s="85"/>
-      <c r="J20" s="112"/>
-      <c r="K20" s="112"/>
+      <c r="J20" s="104"/>
+      <c r="K20" s="104"/>
       <c r="L20" s="84" t="s">
         <v>83</v>
       </c>
@@ -2817,7 +2845,14 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>
-  <mergeCells count="14">
+  <mergeCells count="17">
+    <mergeCell ref="E17:E18"/>
+    <mergeCell ref="J17:K18"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="C6:C7"/>
+    <mergeCell ref="D6:D7"/>
+    <mergeCell ref="E6:E7"/>
     <mergeCell ref="U6:V7"/>
     <mergeCell ref="U10:V10"/>
     <mergeCell ref="J19:K20"/>
@@ -2827,11 +2862,7 @@
     <mergeCell ref="H6:H7"/>
     <mergeCell ref="I6:M6"/>
     <mergeCell ref="N6:R6"/>
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="C6:C7"/>
-    <mergeCell ref="D6:D7"/>
-    <mergeCell ref="E6:E7"/>
+    <mergeCell ref="Q17:R18"/>
   </mergeCells>
   <conditionalFormatting sqref="D8">
     <cfRule type="expression" dxfId="1" priority="8" stopIfTrue="1">

</xml_diff>